<commit_message>
Lagt til utskrift av el- og gas boiler
</commit_message>
<xml_diff>
--- a/Input_data_With_dummyGrid_and_RT_pulp.xlsx
+++ b/Input_data_With_dummyGrid_and_RT_pulp.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Simple_extended\V8\Master_repo\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Simple_extended\Master_repo\Master_repo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE35D3F4-1EA4-478C-984C-EF3E9D8BC619}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{302D1E6E-84DF-4C01-AF49-8F737E4D1A7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="1000" firstSheet="14" activeTab="15" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="1000" firstSheet="7" activeTab="15" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Par_AvailableExcessHeat" sheetId="8" r:id="rId1"/>
@@ -123,7 +123,7 @@
     <author>tc={C5776892-1F20-4F03-80A7-219BD90F0AD8}</author>
   </authors>
   <commentList>
-    <comment ref="C37" authorId="0" shapeId="0" xr:uid="{C5776892-1F20-4F03-80A7-219BD90F0AD8}">
+    <comment ref="C41" authorId="0" shapeId="0" xr:uid="{C5776892-1F20-4F03-80A7-219BD90F0AD8}">
       <text>
         <r>
           <rPr>
@@ -177,7 +177,7 @@
     <author>tc={4AB2F2FD-D9AF-4EF6-975B-D27067AE3E61}</author>
   </authors>
   <commentList>
-    <comment ref="C37" authorId="0" shapeId="0" xr:uid="{4AB2F2FD-D9AF-4EF6-975B-D27067AE3E61}">
+    <comment ref="C41" authorId="0" shapeId="0" xr:uid="{4AB2F2FD-D9AF-4EF6-975B-D27067AE3E61}">
       <text>
         <r>
           <rPr>
@@ -226,7 +226,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="696" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="712" uniqueCount="87">
   <si>
     <t>Benevning:</t>
   </si>
@@ -1564,7 +1564,7 @@
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0E00-000000000000}">
-  <dimension ref="A1:D55"/>
+  <dimension ref="A1:D59"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.42578125" bestFit="1" customWidth="1"/>
@@ -1615,13 +1615,13 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>72</v>
+        <v>60</v>
       </c>
       <c r="B5" t="s">
         <v>28</v>
       </c>
       <c r="C5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D5">
         <v>1</v>
@@ -1629,13 +1629,13 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>73</v>
+        <v>60</v>
       </c>
       <c r="B6" t="s">
         <v>28</v>
       </c>
       <c r="C6">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D6">
         <v>1</v>
@@ -1643,13 +1643,13 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B7" t="s">
         <v>28</v>
       </c>
       <c r="C7">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D7">
         <v>1</v>
@@ -1657,13 +1657,13 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>4</v>
+        <v>72</v>
       </c>
       <c r="B8" t="s">
         <v>28</v>
       </c>
       <c r="C8">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D8">
         <v>1</v>
@@ -1671,10 +1671,10 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>5</v>
+        <v>73</v>
       </c>
       <c r="B9" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C9">
         <v>1</v>
@@ -1685,13 +1685,13 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>61</v>
+        <v>73</v>
       </c>
       <c r="B10" t="s">
-        <v>68</v>
+        <v>28</v>
       </c>
       <c r="C10">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D10">
         <v>1</v>
@@ -1699,13 +1699,13 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>61</v>
+        <v>73</v>
       </c>
       <c r="B11" t="s">
-        <v>68</v>
+        <v>28</v>
       </c>
       <c r="C11">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D11">
         <v>1</v>
@@ -1713,13 +1713,13 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>61</v>
+        <v>4</v>
       </c>
       <c r="B12" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C12">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D12">
         <v>1</v>
@@ -1727,13 +1727,13 @@
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>61</v>
+        <v>5</v>
       </c>
       <c r="B13" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C13">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D13">
         <v>1</v>
@@ -1744,10 +1744,10 @@
         <v>61</v>
       </c>
       <c r="B14" t="s">
-        <v>31</v>
+        <v>68</v>
       </c>
       <c r="C14">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D14">
         <v>1</v>
@@ -1758,10 +1758,10 @@
         <v>61</v>
       </c>
       <c r="B15" t="s">
-        <v>31</v>
+        <v>68</v>
       </c>
       <c r="C15">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D15">
         <v>1</v>
@@ -1769,13 +1769,13 @@
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>78</v>
+        <v>61</v>
       </c>
       <c r="B16" t="s">
-        <v>68</v>
+        <v>30</v>
       </c>
       <c r="C16">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D16">
         <v>1</v>
@@ -1783,13 +1783,13 @@
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>78</v>
+        <v>61</v>
       </c>
       <c r="B17" t="s">
-        <v>68</v>
+        <v>30</v>
       </c>
       <c r="C17">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D17">
         <v>1</v>
@@ -1797,13 +1797,13 @@
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>78</v>
+        <v>61</v>
       </c>
       <c r="B18" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C18">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D18">
         <v>1</v>
@@ -1811,13 +1811,13 @@
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>78</v>
+        <v>61</v>
       </c>
       <c r="B19" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C19">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D19">
         <v>1</v>
@@ -1828,10 +1828,10 @@
         <v>78</v>
       </c>
       <c r="B20" t="s">
-        <v>31</v>
+        <v>68</v>
       </c>
       <c r="C20">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D20">
         <v>1</v>
@@ -1842,10 +1842,10 @@
         <v>78</v>
       </c>
       <c r="B21" t="s">
-        <v>31</v>
+        <v>68</v>
       </c>
       <c r="C21">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D21">
         <v>1</v>
@@ -1853,13 +1853,13 @@
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>62</v>
+        <v>78</v>
       </c>
       <c r="B22" t="s">
-        <v>68</v>
+        <v>30</v>
       </c>
       <c r="C22">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D22">
         <v>1</v>
@@ -1867,13 +1867,13 @@
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>62</v>
+        <v>78</v>
       </c>
       <c r="B23" t="s">
-        <v>68</v>
+        <v>30</v>
       </c>
       <c r="C23">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D23">
         <v>1</v>
@@ -1881,13 +1881,13 @@
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>62</v>
+        <v>78</v>
       </c>
       <c r="B24" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C24">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D24">
         <v>1</v>
@@ -1895,13 +1895,13 @@
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>62</v>
+        <v>78</v>
       </c>
       <c r="B25" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C25">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D25">
         <v>1</v>
@@ -1912,10 +1912,10 @@
         <v>62</v>
       </c>
       <c r="B26" t="s">
-        <v>31</v>
+        <v>68</v>
       </c>
       <c r="C26">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D26">
         <v>1</v>
@@ -1926,10 +1926,10 @@
         <v>62</v>
       </c>
       <c r="B27" t="s">
-        <v>31</v>
+        <v>68</v>
       </c>
       <c r="C27">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D27">
         <v>1</v>
@@ -1937,13 +1937,13 @@
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>77</v>
+        <v>62</v>
       </c>
       <c r="B28" t="s">
-        <v>68</v>
+        <v>30</v>
       </c>
       <c r="C28">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D28">
         <v>1</v>
@@ -1951,13 +1951,13 @@
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>77</v>
+        <v>62</v>
       </c>
       <c r="B29" t="s">
-        <v>68</v>
+        <v>30</v>
       </c>
       <c r="C29">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D29">
         <v>1</v>
@@ -1965,13 +1965,13 @@
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>77</v>
+        <v>62</v>
       </c>
       <c r="B30" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C30">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D30">
         <v>1</v>
@@ -1979,13 +1979,13 @@
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>77</v>
+        <v>62</v>
       </c>
       <c r="B31" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C31">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D31">
         <v>1</v>
@@ -1996,10 +1996,10 @@
         <v>77</v>
       </c>
       <c r="B32" t="s">
-        <v>31</v>
+        <v>68</v>
       </c>
       <c r="C32">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D32">
         <v>1</v>
@@ -2010,135 +2010,185 @@
         <v>77</v>
       </c>
       <c r="B33" t="s">
-        <v>31</v>
+        <v>68</v>
       </c>
       <c r="C33">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D33">
         <v>1</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A34" s="3" t="s">
-        <v>67</v>
+      <c r="A34" t="s">
+        <v>77</v>
       </c>
       <c r="B34" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C34">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D34">
-        <v>0.2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A35" s="3" t="s">
-        <v>67</v>
+      <c r="A35" t="s">
+        <v>77</v>
       </c>
       <c r="B35" t="s">
         <v>30</v>
       </c>
       <c r="C35">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D35">
-        <v>0.8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A36" s="3" t="s">
-        <v>2</v>
+      <c r="A36" t="s">
+        <v>77</v>
       </c>
       <c r="B36" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="C36">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D36">
         <v>1</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A37" s="3" t="s">
-        <v>2</v>
+      <c r="A37" t="s">
+        <v>77</v>
       </c>
       <c r="B37" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="C37">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D37">
         <v>1</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
-        <v>6</v>
+      <c r="A38" s="3" t="s">
+        <v>67</v>
       </c>
       <c r="B38" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C38">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D38">
-        <v>1</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A39" t="s">
-        <v>7</v>
+      <c r="A39" s="3" t="s">
+        <v>67</v>
       </c>
       <c r="B39" t="s">
         <v>30</v>
       </c>
       <c r="C39">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D39">
-        <v>1</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A40" t="s">
+      <c r="A40" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B40" t="s">
+        <v>28</v>
+      </c>
+      <c r="C40">
+        <v>2</v>
+      </c>
+      <c r="D40">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A41" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B41" t="s">
+        <v>28</v>
+      </c>
+      <c r="C41">
+        <v>4</v>
+      </c>
+      <c r="D41">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>6</v>
+      </c>
+      <c r="B42" t="s">
+        <v>31</v>
+      </c>
+      <c r="C42">
+        <v>2</v>
+      </c>
+      <c r="D42">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>7</v>
+      </c>
+      <c r="B43" t="s">
+        <v>30</v>
+      </c>
+      <c r="C43">
+        <v>2</v>
+      </c>
+      <c r="D43">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
         <v>83</v>
       </c>
-      <c r="B40" t="s">
+      <c r="B44" t="s">
         <v>29</v>
       </c>
-      <c r="C40">
-        <v>2</v>
-      </c>
-      <c r="D40">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A41" t="s">
+      <c r="C44">
+        <v>2</v>
+      </c>
+      <c r="D44">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
         <v>86</v>
       </c>
-      <c r="B41" t="s">
+      <c r="B45" t="s">
         <v>85</v>
       </c>
-      <c r="C41">
-        <v>1</v>
-      </c>
-      <c r="D41">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A47" s="3"/>
-    </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A48" s="3"/>
-    </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A49" s="3"/>
+      <c r="C45">
+        <v>1</v>
+      </c>
+      <c r="D45">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="51" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A51" s="3"/>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A52" s="3"/>
@@ -2146,11 +2196,17 @@
     <row r="53" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A53" s="3"/>
     </row>
-    <row r="54" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A54" s="3"/>
-    </row>
-    <row r="55" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A55" s="3"/>
+    <row r="56" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A56" s="3"/>
+    </row>
+    <row r="57" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A57" s="3"/>
+    </row>
+    <row r="58" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A58" s="3"/>
+    </row>
+    <row r="59" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A59" s="3"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
@@ -4720,7 +4776,7 @@
 
 <file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2700-000000000000}">
-  <dimension ref="A3:C55"/>
+  <dimension ref="A3:C59"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="24.42578125" bestFit="1" customWidth="1"/>
@@ -4753,54 +4809,54 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>72</v>
+        <v>60</v>
       </c>
       <c r="B5" t="s">
         <v>28</v>
       </c>
       <c r="C5">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>73</v>
+        <v>60</v>
       </c>
       <c r="B6" t="s">
         <v>28</v>
       </c>
       <c r="C6">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B7" t="s">
         <v>28</v>
       </c>
       <c r="C7">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>4</v>
+        <v>72</v>
       </c>
       <c r="B8" t="s">
         <v>28</v>
       </c>
       <c r="C8">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>5</v>
+        <v>73</v>
       </c>
       <c r="B9" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C9">
         <v>1</v>
@@ -4808,46 +4864,46 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>61</v>
+        <v>73</v>
       </c>
       <c r="B10" t="s">
-        <v>68</v>
+        <v>28</v>
       </c>
       <c r="C10">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>61</v>
+        <v>73</v>
       </c>
       <c r="B11" t="s">
-        <v>68</v>
+        <v>28</v>
       </c>
       <c r="C11">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>61</v>
+        <v>4</v>
       </c>
       <c r="B12" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C12">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>61</v>
+        <v>5</v>
       </c>
       <c r="B13" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C13">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
@@ -4855,10 +4911,10 @@
         <v>61</v>
       </c>
       <c r="B14" t="s">
-        <v>31</v>
+        <v>68</v>
       </c>
       <c r="C14">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
@@ -4866,54 +4922,54 @@
         <v>61</v>
       </c>
       <c r="B15" t="s">
-        <v>31</v>
+        <v>68</v>
       </c>
       <c r="C15">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>78</v>
+        <v>61</v>
       </c>
       <c r="B16" t="s">
-        <v>68</v>
+        <v>30</v>
       </c>
       <c r="C16">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>78</v>
+        <v>61</v>
       </c>
       <c r="B17" t="s">
-        <v>68</v>
+        <v>30</v>
       </c>
       <c r="C17">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>78</v>
+        <v>61</v>
       </c>
       <c r="B18" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C18">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>78</v>
+        <v>61</v>
       </c>
       <c r="B19" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C19">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
@@ -4921,10 +4977,10 @@
         <v>78</v>
       </c>
       <c r="B20" t="s">
-        <v>31</v>
+        <v>68</v>
       </c>
       <c r="C20">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
@@ -4932,54 +4988,54 @@
         <v>78</v>
       </c>
       <c r="B21" t="s">
-        <v>31</v>
+        <v>68</v>
       </c>
       <c r="C21">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>62</v>
+        <v>78</v>
       </c>
       <c r="B22" t="s">
-        <v>68</v>
+        <v>30</v>
       </c>
       <c r="C22">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>62</v>
+        <v>78</v>
       </c>
       <c r="B23" t="s">
-        <v>68</v>
+        <v>30</v>
       </c>
       <c r="C23">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>62</v>
+        <v>78</v>
       </c>
       <c r="B24" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C24">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>62</v>
+        <v>78</v>
       </c>
       <c r="B25" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C25">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
@@ -4987,10 +5043,10 @@
         <v>62</v>
       </c>
       <c r="B26" t="s">
-        <v>31</v>
+        <v>68</v>
       </c>
       <c r="C26">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
@@ -4998,54 +5054,54 @@
         <v>62</v>
       </c>
       <c r="B27" t="s">
-        <v>31</v>
+        <v>68</v>
       </c>
       <c r="C27">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>77</v>
+        <v>62</v>
       </c>
       <c r="B28" t="s">
-        <v>68</v>
+        <v>30</v>
       </c>
       <c r="C28">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>77</v>
+        <v>62</v>
       </c>
       <c r="B29" t="s">
-        <v>68</v>
+        <v>30</v>
       </c>
       <c r="C29">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>77</v>
+        <v>62</v>
       </c>
       <c r="B30" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C30">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>77</v>
+        <v>62</v>
       </c>
       <c r="B31" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C31">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
@@ -5053,10 +5109,10 @@
         <v>77</v>
       </c>
       <c r="B32" t="s">
-        <v>31</v>
+        <v>68</v>
       </c>
       <c r="C32">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
@@ -5064,84 +5120,84 @@
         <v>77</v>
       </c>
       <c r="B33" t="s">
-        <v>31</v>
+        <v>68</v>
       </c>
       <c r="C33">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A34" s="3" t="s">
-        <v>67</v>
+      <c r="A34" t="s">
+        <v>77</v>
       </c>
       <c r="B34" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C34">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A35" s="3" t="s">
-        <v>67</v>
+      <c r="A35" t="s">
+        <v>77</v>
       </c>
       <c r="B35" t="s">
         <v>30</v>
       </c>
       <c r="C35">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A36" s="3" t="s">
-        <v>2</v>
+      <c r="A36" t="s">
+        <v>77</v>
       </c>
       <c r="B36" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="C36">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A37" s="3" t="s">
-        <v>2</v>
+      <c r="A37" t="s">
+        <v>77</v>
       </c>
       <c r="B37" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="C37">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
-        <v>6</v>
+      <c r="A38" s="3" t="s">
+        <v>67</v>
       </c>
       <c r="B38" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C38">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A39" t="s">
-        <v>7</v>
+      <c r="A39" s="3" t="s">
+        <v>67</v>
       </c>
       <c r="B39" t="s">
         <v>30</v>
       </c>
       <c r="C39">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" s="3" t="s">
-        <v>83</v>
+        <v>2</v>
       </c>
       <c r="B40" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C40">
         <v>2</v>
@@ -5149,23 +5205,61 @@
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B41" t="s">
+        <v>28</v>
+      </c>
+      <c r="C41">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>6</v>
+      </c>
+      <c r="B42" t="s">
+        <v>31</v>
+      </c>
+      <c r="C42">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>7</v>
+      </c>
+      <c r="B43" t="s">
+        <v>30</v>
+      </c>
+      <c r="C43">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A44" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="B44" t="s">
+        <v>29</v>
+      </c>
+      <c r="C44">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A45" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="B41" t="s">
+      <c r="B45" t="s">
         <v>85</v>
       </c>
-      <c r="C41">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A47" s="3"/>
-    </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A48" s="3"/>
-    </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A49" s="3"/>
+      <c r="C45">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="51" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A51" s="3"/>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A52" s="3"/>
@@ -5173,11 +5267,17 @@
     <row r="53" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A53" s="3"/>
     </row>
-    <row r="54" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A54" s="3"/>
-    </row>
-    <row r="55" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A55" s="3"/>
+    <row r="56" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A56" s="3"/>
+    </row>
+    <row r="57" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A57" s="3"/>
+    </row>
+    <row r="58" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A58" s="3"/>
+    </row>
+    <row r="59" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A59" s="3"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>

</xml_diff>